<commit_message>
csv handle incomplete or empty rows + tests
</commit_message>
<xml_diff>
--- a/tests/TestData.xlsx
+++ b/tests/TestData.xlsx
@@ -808,10 +808,10 @@
       <c r="B5" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E5" t="s">
@@ -924,45 +924,60 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="s">
+      <c r="A10" s="2"/>
+      <c r="B10"/>
+      <c r="C10"/>
+      <c r="D10"/>
+      <c r="E10" s="2"/>
+      <c r="F10"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2"/>
+      <c r="B11"/>
+      <c r="C11"/>
+      <c r="D11"/>
+      <c r="E11" s="2"/>
+      <c r="F11"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2"/>
+      <c r="B12"/>
+      <c r="C12"/>
+      <c r="D12"/>
+      <c r="E12" s="2"/>
+      <c r="F12"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
         <v>54</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B13" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" t="s">
-        <v>56</v>
-      </c>
-      <c r="F10" s="1"/>
-      <c r="G10" t="s">
-        <v>57</v>
-      </c>
-      <c r="H10" t="s">
-        <v>58</v>
-      </c>
-      <c r="I10">
-        <v>94086</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="F11" s="1"/>
-    </row>
-    <row r="12">
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="F12" s="1"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
+      <c r="E13" t="s">
+        <v>56</v>
+      </c>
       <c r="F13" s="1"/>
+      <c r="G13" t="s">
+        <v>57</v>
+      </c>
+      <c r="H13" t="s">
+        <v>58</v>
+      </c>
+      <c r="I13">
+        <v>94086</v>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="1"/>
@@ -994,8 +1009,26 @@
       <c r="D18" s="1"/>
       <c r="F18" s="1"/>
     </row>
-    <row r="22" ht="14.25">
-      <c r="F22" s="1"/>
+    <row r="19">
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="F19" s="1"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="F20" s="1"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="F21" s="1"/>
+    </row>
+    <row r="25" ht="14.25">
+      <c r="F25" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>